<commit_message>
ver.0.4.2.1 DT is converted to kable
</commit_message>
<xml_diff>
--- a/data/chapter34_Rmarkdown.xlsx
+++ b/data/chapter34_Rmarkdown.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\araya\Documents\R入門\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\R入門\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AF71ABBD-1DA2-4547-AE04-442A55EB7C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA3A116-5F83-4DF3-8275-C75098BF1658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{45AADD67-DB4F-41EA-A38B-1FE6C1AF3A60}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="19410" windowHeight="16305" xr2:uid="{45AADD67-DB4F-41EA-A38B-1FE6C1AF3A60}"/>
   </bookViews>
   <sheets>
     <sheet name="markdown" sheetId="1" r:id="rId1"/>
@@ -40,18 +40,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="115">
   <si>
-    <t>_text_</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>*text*</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>**text**</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>イタリック</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -63,10 +51,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>~text~</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>下付き</t>
     <rPh sb="0" eb="2">
       <t>シタツ</t>
@@ -74,10 +58,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>^text^</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>上付き</t>
     <rPh sb="0" eb="2">
       <t>ウエツ</t>
@@ -85,10 +65,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>```code```</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>スクリプト表記</t>
     <rPh sb="5" eb="7">
       <t>ヒョウキ</t>
@@ -103,21 +79,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>```` ```code``` ````</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>```を表示（```code```）</t>
-    <rPh sb="4" eb="6">
-      <t>ヒョウジ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>[text](address)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>リンク</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -132,10 +93,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>^[text]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>脚注（foot note）</t>
     <rPh sb="0" eb="2">
       <t>キャクチュウ</t>
@@ -143,10 +100,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>[@bibtex]</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>文献の参照</t>
     <rPh sb="0" eb="2">
       <t>ブンケン</t>
@@ -226,10 +179,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>$$ math $$</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>LaTeXの数式</t>
     <rPh sb="6" eb="8">
       <t>スウシキ</t>
@@ -248,17 +197,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>![text](path_to_image)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>`r code`</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>`code`</t>
-  </si>
-  <si>
     <t>スクリプト表記（インライン）</t>
     <rPh sb="5" eb="7">
       <t>ヒョウキ</t>
@@ -721,6 +659,69 @@
     </rPh>
     <rPh sb="6" eb="8">
       <t>セッテイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\_text\_</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\*text\*</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\**text\**</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\~text\~</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\^tex\t^</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\`code\`</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\`\`\`\`\`\`\`code\`\`\`\`\`\`\`</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\!\[text\]\(path_to_image\)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\[text\]\(address\)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\^\[text\]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\[\@bibtex\]</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\$$ math \$$</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\`r code\`</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\`\`\`code\`\`\`</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>\`\`\`を表示（\`\`\`code\`\`\`）</t>
+    <rPh sb="7" eb="9">
+      <t>ヒョウジ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -1118,194 +1119,194 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" t="s">
         <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>102</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>103</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>105</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>112</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>106</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>108</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>107</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>109</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>110</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A18" s="1" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A19" s="1" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A20" s="1" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A23" s="1" t="s">
-        <v>35</v>
+        <v>111</v>
       </c>
       <c r="B23" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A24" s="1" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1326,189 +1327,189 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" t="s">
         <v>64</v>
-      </c>
-      <c r="C2" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="C9" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C15" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1527,106 +1528,106 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="B6" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="B7" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="B9" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B10" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="B11" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>